<commit_message>
Add public/llms.txt for AI/GEO readiness
Fixes SEO audit finding #3 — NordPush explicitly sells GEO-Optimierung
as a service, so the missing llms.txt was a positioning inconsistency.

Content covers the full site hierarchy: 5 website types, 22 SEO
service pages, all 3 pricing models (Cash / Abo / Bundle) with prices,
agency info, knowledge section, legal, and contact details.

Also updates the audit Excel: findings #3 marked "Behoben",
counters in Zusammenfassung reflect new status.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NordPush-SEO-Audit-2026-04-23.xlsx
+++ b/NordPush-SEO-Audit-2026-04-23.xlsx
@@ -682,8 +682,10 @@
           <t>Hoher Impact</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n">
-        <v>3</v>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>3 (1 behoben, 2 offen)</t>
+        </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -906,9 +908,9 @@
       <c r="H4" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>Offen</t>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>Behoben</t>
         </is>
       </c>
     </row>

</xml_diff>